<commit_message>
deploy: feature/careteam → branches/feature-careteam 079854d906938ded8df3eae1e7f7bfc9b2b1bc72
</commit_message>
<xml_diff>
--- a/branches/feature-careteam/StructureDefinition-contact-point-availability.xlsx
+++ b/branches/feature-careteam/StructureDefinition-contact-point-availability.xlsx
@@ -10,13 +10,13 @@
     <sheet name="Elements" r:id="rId4" sheetId="2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AK$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AK$21</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="699" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="734" uniqueCount="180">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-10-15T14:04:45+00:00</t>
+    <t>2026-10-28T12:18:22+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -344,7 +344,7 @@
     <t>Kontaktvägens tillgänglighet</t>
   </si>
   <si>
-    <t>Anger under vilka veckodagar och tider kontaktvägen är tillgänglig.</t>
+    <t>Value of extension - must be one of a constrained set of the data types (see [Extensibility](http://hl7.org/fhir/R5/extensibility.html) for a list).</t>
   </si>
   <si>
     <t xml:space="preserve">ext-1
@@ -387,6 +387,9 @@
     <t>Anger återkommande veckodagar och tider då kontaktvägen är tillgänglig.</t>
   </si>
   <si>
+    <t>Saknas veckodagar, tider och period är kontaktvägen tillgänglig alla dagar, hela dygnet, tills vidare.</t>
+  </si>
+  <si>
     <t>A collection of times that the {item} is available.</t>
   </si>
   <si>
@@ -407,6 +410,22 @@
     <t>Extension.value[x].availableTime.extension</t>
   </si>
   <si>
+    <t>Extension.value[x].availableTime.extension:period</t>
+  </si>
+  <si>
+    <t>period</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Extension {https://fhir.inera.se/ig/careteam/StructureDefinition/available-time-period}
+</t>
+  </si>
+  <si>
+    <t>Period</t>
+  </si>
+  <si>
+    <t>Datumperiod under vilken veckodagarna och tiderna gäller. Saknas perioden gäller tiderna tills vidare.</t>
+  </si>
+  <si>
     <t>Extension.value[x].availableTime.daysOfWeek</t>
   </si>
   <si>
@@ -420,6 +439,9 @@
     <t>Veckodag då kontaktvägen är tillgänglig.</t>
   </si>
   <si>
+    <t>Saknas veckodag gäller tiderna alla dagar i veckan.</t>
+  </si>
+  <si>
     <t>Indicates which days of the week are available between the start and end Times.</t>
   </si>
   <si>
@@ -471,7 +493,7 @@
     <t>Tidpunkt då tillgängligheten börjar.</t>
   </si>
   <si>
-    <t>The timezone is expected to be specified or implied by the context this datatype is used.</t>
+    <t>Saknas starttid gäller tillgängligheten från dagens början.</t>
   </si>
   <si>
     <t>The opening time of day. Note: If the AllDay flag is set, then this time is ignored.</t>
@@ -487,6 +509,9 @@
   </si>
   <si>
     <t>Tidpunkt då tillgängligheten upphör.</t>
+  </si>
+  <si>
+    <t>Saknas sluttid gäller tillgängligheten till dagens slut.</t>
   </si>
   <si>
     <t>The closing time of day. Note: If the AllDay flag is set, then this time is ignored.</t>
@@ -876,7 +901,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AK20"/>
+  <dimension ref="A1:AK21"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="42.37890625" customWidth="true" bestFit="true"/>
@@ -889,7 +914,7 @@
     <col min="8" max="8" width="13.953125" customWidth="true" bestFit="true"/>
     <col min="9" max="9" width="11.3671875" customWidth="true" bestFit="true"/>
     <col min="10" max="10" width="20.703125" customWidth="true" bestFit="true"/>
-    <col min="11" max="11" width="9.5546875" customWidth="true" bestFit="true"/>
+    <col min="11" max="11" width="68.984375" customWidth="true" bestFit="true"/>
     <col min="12" max="12" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="13" max="13" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="14" max="14" width="100.703125" customWidth="true" bestFit="true"/>
@@ -1791,9 +1816,11 @@
       <c r="M9" t="s" s="2">
         <v>118</v>
       </c>
-      <c r="N9" s="2"/>
+      <c r="N9" t="s" s="2">
+        <v>119</v>
+      </c>
       <c r="O9" t="s" s="2">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="P9" t="s" s="2">
         <v>76</v>
@@ -1842,7 +1869,7 @@
         <v>76</v>
       </c>
       <c r="AF9" t="s" s="2">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="AG9" t="s" s="2">
         <v>77</v>
@@ -1854,7 +1881,7 @@
         <v>76</v>
       </c>
       <c r="AJ9" t="s" s="2">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="AK9" t="s" s="2">
         <v>76</v>
@@ -1862,10 +1889,10 @@
     </row>
     <row r="10" hidden="true">
       <c r="A10" t="s" s="2">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B10" t="s" s="2">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C10" s="2"/>
       <c r="D10" t="s" s="2">
@@ -1888,7 +1915,7 @@
         <v>76</v>
       </c>
       <c r="K10" t="s" s="2">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="L10" t="s" s="2">
         <v>84</v>
@@ -1965,10 +1992,10 @@
     </row>
     <row r="11" hidden="true">
       <c r="A11" t="s" s="2">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B11" t="s" s="2">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" t="s" s="2">
@@ -2070,21 +2097,23 @@
     </row>
     <row r="12">
       <c r="A12" t="s" s="2">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B12" t="s" s="2">
         <v>125</v>
       </c>
-      <c r="C12" s="2"/>
+      <c r="C12" t="s" s="2">
+        <v>127</v>
+      </c>
       <c r="D12" t="s" s="2">
         <v>76</v>
       </c>
       <c r="E12" s="2"/>
       <c r="F12" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="G12" t="s" s="2">
         <v>82</v>
-      </c>
-      <c r="G12" t="s" s="2">
-        <v>78</v>
       </c>
       <c r="H12" t="s" s="2">
         <v>103</v>
@@ -2093,21 +2122,19 @@
         <v>76</v>
       </c>
       <c r="J12" t="s" s="2">
-        <v>103</v>
+        <v>76</v>
       </c>
       <c r="K12" t="s" s="2">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="L12" t="s" s="2">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="M12" t="s" s="2">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="N12" s="2"/>
-      <c r="O12" t="s" s="2">
-        <v>129</v>
-      </c>
+      <c r="O12" s="2"/>
       <c r="P12" t="s" s="2">
         <v>76</v>
       </c>
@@ -2131,13 +2158,13 @@
         <v>76</v>
       </c>
       <c r="X12" t="s" s="2">
-        <v>130</v>
+        <v>76</v>
       </c>
       <c r="Y12" t="s" s="2">
-        <v>131</v>
+        <v>76</v>
       </c>
       <c r="Z12" t="s" s="2">
-        <v>132</v>
+        <v>76</v>
       </c>
       <c r="AA12" t="s" s="2">
         <v>76</v>
@@ -2155,7 +2182,7 @@
         <v>76</v>
       </c>
       <c r="AF12" t="s" s="2">
-        <v>133</v>
+        <v>95</v>
       </c>
       <c r="AG12" t="s" s="2">
         <v>77</v>
@@ -2167,18 +2194,18 @@
         <v>76</v>
       </c>
       <c r="AJ12" t="s" s="2">
-        <v>108</v>
+        <v>80</v>
       </c>
       <c r="AK12" t="s" s="2">
         <v>76</v>
       </c>
     </row>
-    <row r="13" hidden="true">
+    <row r="13">
       <c r="A13" t="s" s="2">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="B13" t="s" s="2">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" t="s" s="2">
@@ -2186,13 +2213,13 @@
       </c>
       <c r="E13" s="2"/>
       <c r="F13" t="s" s="2">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="G13" t="s" s="2">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="H13" t="s" s="2">
-        <v>76</v>
+        <v>103</v>
       </c>
       <c r="I13" t="s" s="2">
         <v>76</v>
@@ -2201,17 +2228,19 @@
         <v>103</v>
       </c>
       <c r="K13" t="s" s="2">
+        <v>132</v>
+      </c>
+      <c r="L13" t="s" s="2">
+        <v>133</v>
+      </c>
+      <c r="M13" t="s" s="2">
+        <v>134</v>
+      </c>
+      <c r="N13" t="s" s="2">
         <v>135</v>
       </c>
-      <c r="L13" t="s" s="2">
+      <c r="O13" t="s" s="2">
         <v>136</v>
-      </c>
-      <c r="M13" t="s" s="2">
-        <v>137</v>
-      </c>
-      <c r="N13" s="2"/>
-      <c r="O13" t="s" s="2">
-        <v>138</v>
       </c>
       <c r="P13" t="s" s="2">
         <v>76</v>
@@ -2236,13 +2265,13 @@
         <v>76</v>
       </c>
       <c r="X13" t="s" s="2">
-        <v>76</v>
+        <v>137</v>
       </c>
       <c r="Y13" t="s" s="2">
-        <v>76</v>
+        <v>138</v>
       </c>
       <c r="Z13" t="s" s="2">
-        <v>76</v>
+        <v>139</v>
       </c>
       <c r="AA13" t="s" s="2">
         <v>76</v>
@@ -2260,16 +2289,16 @@
         <v>76</v>
       </c>
       <c r="AF13" t="s" s="2">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="AG13" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH13" t="s" s="2">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="AI13" t="s" s="2">
-        <v>140</v>
+        <v>76</v>
       </c>
       <c r="AJ13" t="s" s="2">
         <v>108</v>
@@ -2278,7 +2307,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" hidden="true">
       <c r="A14" t="s" s="2">
         <v>141</v>
       </c>
@@ -2297,7 +2326,7 @@
         <v>82</v>
       </c>
       <c r="H14" t="s" s="2">
-        <v>103</v>
+        <v>76</v>
       </c>
       <c r="I14" t="s" s="2">
         <v>76</v>
@@ -2314,11 +2343,9 @@
       <c r="M14" t="s" s="2">
         <v>144</v>
       </c>
-      <c r="N14" t="s" s="2">
+      <c r="N14" s="2"/>
+      <c r="O14" t="s" s="2">
         <v>145</v>
-      </c>
-      <c r="O14" t="s" s="2">
-        <v>146</v>
       </c>
       <c r="P14" t="s" s="2">
         <v>76</v>
@@ -2367,7 +2394,7 @@
         <v>76</v>
       </c>
       <c r="AF14" t="s" s="2">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="AG14" t="s" s="2">
         <v>77</v>
@@ -2376,7 +2403,7 @@
         <v>82</v>
       </c>
       <c r="AI14" t="s" s="2">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="AJ14" t="s" s="2">
         <v>108</v>
@@ -2413,19 +2440,19 @@
         <v>103</v>
       </c>
       <c r="K15" t="s" s="2">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="L15" t="s" s="2">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="M15" t="s" s="2">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="N15" t="s" s="2">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="O15" t="s" s="2">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="P15" t="s" s="2">
         <v>76</v>
@@ -2474,7 +2501,7 @@
         <v>76</v>
       </c>
       <c r="AF15" t="s" s="2">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="AG15" t="s" s="2">
         <v>77</v>
@@ -2483,7 +2510,7 @@
         <v>82</v>
       </c>
       <c r="AI15" t="s" s="2">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="AJ15" t="s" s="2">
         <v>108</v>
@@ -2492,12 +2519,12 @@
         <v>76</v>
       </c>
     </row>
-    <row r="16" hidden="true">
+    <row r="16">
       <c r="A16" t="s" s="2">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B16" t="s" s="2">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" t="s" s="2">
@@ -2508,10 +2535,10 @@
         <v>77</v>
       </c>
       <c r="G16" t="s" s="2">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="H16" t="s" s="2">
-        <v>76</v>
+        <v>103</v>
       </c>
       <c r="I16" t="s" s="2">
         <v>76</v>
@@ -2520,17 +2547,19 @@
         <v>103</v>
       </c>
       <c r="K16" t="s" s="2">
-        <v>116</v>
+        <v>149</v>
       </c>
       <c r="L16" t="s" s="2">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="M16" t="s" s="2">
-        <v>155</v>
-      </c>
-      <c r="N16" s="2"/>
+        <v>157</v>
+      </c>
+      <c r="N16" t="s" s="2">
+        <v>158</v>
+      </c>
       <c r="O16" t="s" s="2">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="P16" t="s" s="2">
         <v>76</v>
@@ -2579,16 +2608,16 @@
         <v>76</v>
       </c>
       <c r="AF16" t="s" s="2">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="AG16" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH16" t="s" s="2">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="AI16" t="s" s="2">
-        <v>76</v>
+        <v>147</v>
       </c>
       <c r="AJ16" t="s" s="2">
         <v>108</v>
@@ -2599,10 +2628,10 @@
     </row>
     <row r="17" hidden="true">
       <c r="A17" t="s" s="2">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="B17" t="s" s="2">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" t="s" s="2">
@@ -2613,7 +2642,7 @@
         <v>77</v>
       </c>
       <c r="G17" t="s" s="2">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="H17" t="s" s="2">
         <v>76</v>
@@ -2622,19 +2651,21 @@
         <v>76</v>
       </c>
       <c r="J17" t="s" s="2">
-        <v>76</v>
+        <v>103</v>
       </c>
       <c r="K17" t="s" s="2">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="L17" t="s" s="2">
-        <v>84</v>
+        <v>162</v>
       </c>
       <c r="M17" t="s" s="2">
-        <v>85</v>
+        <v>163</v>
       </c>
       <c r="N17" s="2"/>
-      <c r="O17" s="2"/>
+      <c r="O17" t="s" s="2">
+        <v>164</v>
+      </c>
       <c r="P17" t="s" s="2">
         <v>76</v>
       </c>
@@ -2682,41 +2713,41 @@
         <v>76</v>
       </c>
       <c r="AF17" t="s" s="2">
-        <v>86</v>
+        <v>165</v>
       </c>
       <c r="AG17" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH17" t="s" s="2">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="AI17" t="s" s="2">
-        <v>87</v>
+        <v>76</v>
       </c>
       <c r="AJ17" t="s" s="2">
-        <v>76</v>
+        <v>108</v>
       </c>
       <c r="AK17" t="s" s="2">
-        <v>88</v>
+        <v>76</v>
       </c>
     </row>
     <row r="18" hidden="true">
       <c r="A18" t="s" s="2">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="B18" t="s" s="2">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" t="s" s="2">
-        <v>111</v>
+        <v>76</v>
       </c>
       <c r="E18" s="2"/>
       <c r="F18" t="s" s="2">
         <v>77</v>
       </c>
       <c r="G18" t="s" s="2">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="H18" t="s" s="2">
         <v>76</v>
@@ -2728,17 +2759,15 @@
         <v>76</v>
       </c>
       <c r="K18" t="s" s="2">
-        <v>90</v>
+        <v>124</v>
       </c>
       <c r="L18" t="s" s="2">
-        <v>112</v>
+        <v>84</v>
       </c>
       <c r="M18" t="s" s="2">
-        <v>113</v>
-      </c>
-      <c r="N18" t="s" s="2">
-        <v>114</v>
-      </c>
+        <v>85</v>
+      </c>
+      <c r="N18" s="2"/>
       <c r="O18" s="2"/>
       <c r="P18" t="s" s="2">
         <v>76</v>
@@ -2775,31 +2804,31 @@
         <v>76</v>
       </c>
       <c r="AB18" t="s" s="2">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="AC18" t="s" s="2">
-        <v>93</v>
+        <v>76</v>
       </c>
       <c r="AD18" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AE18" t="s" s="2">
-        <v>94</v>
+        <v>76</v>
       </c>
       <c r="AF18" t="s" s="2">
-        <v>95</v>
+        <v>86</v>
       </c>
       <c r="AG18" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH18" t="s" s="2">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="AI18" t="s" s="2">
-        <v>76</v>
+        <v>87</v>
       </c>
       <c r="AJ18" t="s" s="2">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="AK18" t="s" s="2">
         <v>88</v>
@@ -2807,21 +2836,21 @@
     </row>
     <row r="19" hidden="true">
       <c r="A19" t="s" s="2">
-        <v>160</v>
+        <v>167</v>
       </c>
       <c r="B19" t="s" s="2">
-        <v>160</v>
+        <v>167</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" t="s" s="2">
-        <v>76</v>
+        <v>111</v>
       </c>
       <c r="E19" s="2"/>
       <c r="F19" t="s" s="2">
         <v>77</v>
       </c>
       <c r="G19" t="s" s="2">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="H19" t="s" s="2">
         <v>76</v>
@@ -2830,23 +2859,21 @@
         <v>76</v>
       </c>
       <c r="J19" t="s" s="2">
-        <v>103</v>
+        <v>76</v>
       </c>
       <c r="K19" t="s" s="2">
-        <v>123</v>
+        <v>90</v>
       </c>
       <c r="L19" t="s" s="2">
-        <v>161</v>
+        <v>112</v>
       </c>
       <c r="M19" t="s" s="2">
-        <v>162</v>
+        <v>113</v>
       </c>
       <c r="N19" t="s" s="2">
-        <v>163</v>
-      </c>
-      <c r="O19" t="s" s="2">
-        <v>164</v>
-      </c>
+        <v>114</v>
+      </c>
+      <c r="O19" s="2"/>
       <c r="P19" t="s" s="2">
         <v>76</v>
       </c>
@@ -2882,42 +2909,42 @@
         <v>76</v>
       </c>
       <c r="AB19" t="s" s="2">
-        <v>76</v>
+        <v>92</v>
       </c>
       <c r="AC19" t="s" s="2">
-        <v>76</v>
+        <v>93</v>
       </c>
       <c r="AD19" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AE19" t="s" s="2">
-        <v>76</v>
+        <v>94</v>
       </c>
       <c r="AF19" t="s" s="2">
-        <v>165</v>
+        <v>95</v>
       </c>
       <c r="AG19" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH19" t="s" s="2">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="AI19" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ19" t="s" s="2">
-        <v>108</v>
+        <v>80</v>
       </c>
       <c r="AK19" t="s" s="2">
-        <v>76</v>
+        <v>88</v>
       </c>
     </row>
     <row r="20" hidden="true">
       <c r="A20" t="s" s="2">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B20" t="s" s="2">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" t="s" s="2">
@@ -2940,17 +2967,19 @@
         <v>103</v>
       </c>
       <c r="K20" t="s" s="2">
-        <v>167</v>
+        <v>124</v>
       </c>
       <c r="L20" t="s" s="2">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="M20" t="s" s="2">
-        <v>169</v>
-      </c>
-      <c r="N20" s="2"/>
+        <v>170</v>
+      </c>
+      <c r="N20" t="s" s="2">
+        <v>171</v>
+      </c>
       <c r="O20" t="s" s="2">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="P20" t="s" s="2">
         <v>76</v>
@@ -2999,7 +3028,7 @@
         <v>76</v>
       </c>
       <c r="AF20" t="s" s="2">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="AG20" t="s" s="2">
         <v>77</v>
@@ -3017,8 +3046,113 @@
         <v>76</v>
       </c>
     </row>
+    <row r="21" hidden="true">
+      <c r="A21" t="s" s="2">
+        <v>174</v>
+      </c>
+      <c r="B21" t="s" s="2">
+        <v>174</v>
+      </c>
+      <c r="C21" s="2"/>
+      <c r="D21" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="E21" s="2"/>
+      <c r="F21" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="G21" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="H21" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="I21" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="J21" t="s" s="2">
+        <v>103</v>
+      </c>
+      <c r="K21" t="s" s="2">
+        <v>175</v>
+      </c>
+      <c r="L21" t="s" s="2">
+        <v>176</v>
+      </c>
+      <c r="M21" t="s" s="2">
+        <v>177</v>
+      </c>
+      <c r="N21" s="2"/>
+      <c r="O21" t="s" s="2">
+        <v>178</v>
+      </c>
+      <c r="P21" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Q21" s="2"/>
+      <c r="R21" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="S21" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="T21" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="U21" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="V21" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="W21" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="X21" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Y21" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Z21" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AA21" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AB21" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AC21" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AD21" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AE21" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AF21" t="s" s="2">
+        <v>179</v>
+      </c>
+      <c r="AG21" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH21" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AI21" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AJ21" t="s" s="2">
+        <v>108</v>
+      </c>
+      <c r="AK21" t="s" s="2">
+        <v>76</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AK20">
+  <autoFilter ref="A1:AK21">
     <filterColumn colId="7">
       <customFilters>
         <customFilter operator="notEqual" val=" "/>
@@ -3028,7 +3162,7 @@
       <filters blank="true"/>
     </filterColumn>
   </autoFilter>
-  <conditionalFormatting sqref="A2:AI19">
+  <conditionalFormatting sqref="A2:AI20">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>$G2&lt;&gt;"Y"</formula>
     </cfRule>

</xml_diff>